<commit_message>
Quotes cut at the end drop the comma or semicolon before the final … (15 thoughts); rule in DECISIONS, change log in exports/
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/thoughts.xlsx
+++ b/content/thoughts.xlsx
@@ -2638,7 +2638,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Time is like a river made up of the events which happen, and a violent stream; …</t>
+          <t>Time is like a river made up of the events which happen, and a violent stream …</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Love the art, poor as it may be, which you have learned, and be content with it; …</t>
+          <t>Love the art, poor as it may be, which you have learned, and be content with it …</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Constantly regard the universe as one living being, having one substance and one soul; …</t>
+          <t>Constantly regard the universe as one living being, having one substance and one soul …</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>For man, when perfected, is the best of animals, but, when separated from law and justice, he is the worst of all; …</t>
+          <t>For man, when perfected, is the best of animals, but, when separated from law and justice, he is the worst of all …</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
@@ -16599,7 +16599,7 @@
       </c>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>Cheerfulness is a direct and immediate gain,—the very coin, as it were, of happiness, …</t>
+          <t>Cheerfulness is a direct and immediate gain,—the very coin, as it were, of happiness …</t>
         </is>
       </c>
       <c r="C254" s="4" t="inlineStr">
@@ -19332,7 +19332,7 @@
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>If I can stop one heart from breaking, / I shall not live in vain; …</t>
+          <t>If I can stop one heart from breaking, / I shall not live in vain …</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
@@ -19458,7 +19458,7 @@
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>Much madness is divinest sense / To a discerning eye; …</t>
+          <t>Much madness is divinest sense / To a discerning eye …</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
@@ -19769,7 +19769,7 @@
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>To divert myself from a troublesome fancy, 'tis but to run to my books; …</t>
+          <t>To divert myself from a troublesome fancy, 'tis but to run to my books …</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr">
@@ -26322,7 +26322,7 @@
       </c>
       <c r="B407" s="4" t="inlineStr">
         <is>
-          <t>He works best who works without any motive, neither for money, nor for fame, nor for anything else; …</t>
+          <t>He works best who works without any motive, neither for money, nor for fame, nor for anything else …</t>
         </is>
       </c>
       <c r="C407" s="4" t="inlineStr">
@@ -26385,7 +26385,7 @@
       </c>
       <c r="B408" s="4" t="inlineStr">
         <is>
-          <t>Let us do good because it is good to do good; …</t>
+          <t>Let us do good because it is good to do good …</t>
         </is>
       </c>
       <c r="C408" s="4" t="inlineStr">
@@ -26507,7 +26507,7 @@
       </c>
       <c r="B410" s="4" t="inlineStr">
         <is>
-          <t>The true prevails, not the untrue; …</t>
+          <t>The true prevails, not the untrue …</t>
         </is>
       </c>
       <c r="C410" s="4" t="inlineStr">
@@ -28697,7 +28697,7 @@
       </c>
       <c r="B444" s="4" t="inlineStr">
         <is>
-          <t>He who stands on his tiptoes does not stand firm; he who stretches his legs does not walk easily. So, he who displays himself does not shine; he who asserts his own views is not distinguished; …</t>
+          <t>He who stands on his tiptoes does not stand firm; he who stretches his legs does not walk easily. So, he who displays himself does not shine; he who asserts his own views is not distinguished …</t>
         </is>
       </c>
       <c r="C444" s="4" t="inlineStr">
@@ -28945,7 +28945,7 @@
       </c>
       <c r="B448" s="4" t="inlineStr">
         <is>
-          <t>Therefore the sage puts his own person last, and yet it is found in the foremost place; …</t>
+          <t>Therefore the sage puts his own person last, and yet it is found in the foremost place …</t>
         </is>
       </c>
       <c r="C448" s="4" t="inlineStr">
@@ -29197,7 +29197,7 @@
       </c>
       <c r="B452" s="4" t="inlineStr">
         <is>
-          <t>Favour and disgrace would seem equally to be feared; …</t>
+          <t>Favour and disgrace would seem equally to be feared …</t>
         </is>
       </c>
       <c r="C452" s="4" t="inlineStr">
@@ -38460,7 +38460,7 @@
       </c>
       <c r="B598" s="4" t="inlineStr">
         <is>
-          <t>Saying this one is my enemy, and this one my foe, / While it is his own body which is his enemy and foe, …</t>
+          <t>Saying this one is my enemy, and this one my foe, / While it is his own body which is his enemy and foe …</t>
         </is>
       </c>
       <c r="C598" s="4" t="inlineStr">

</xml_diff>